<commit_message>
add the feedforward network
</commit_message>
<xml_diff>
--- a/data/cv_accuracy_all.xlsx
+++ b/data/cv_accuracy_all.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,7 +455,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9619047619047619</v>
+        <v>0.7803030303030303</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8857142857142857</v>
+        <v>0.7651515151515151</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.7954545454545454</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.8409090909090909</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9711538461538461</v>
+        <v>0.8702290076335878</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8761904761904762</v>
+        <v>0.7272727272727273</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7904761904761904</v>
+        <v>0.7954545454545454</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8653846153846154</v>
+        <v>0.803030303030303</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +559,7 @@
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8269230769230769</v>
+        <v>0.7121212121212122</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,72 @@
         <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8269230769230769</v>
+        <v>0.7557251908396947</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>hypothalamus</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.6590909090909091</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>hypothalamus</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.7348484848484849</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>hypothalamus</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>hypothalamus</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.7651515151515151</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>hypothalamus</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.7633587786259542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>